<commit_message>
feat : AStar 이동로직
</commit_message>
<xml_diff>
--- a/Assets/Excels/CreatureSheet.xlsx
+++ b/Assets/Excels/CreatureSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Devs\ProjectD\Assets\Excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3955802-1335-4E17-9416-8321C0FDAF4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1E46695-1AEB-4D78-9D38-21EE46E857C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{BE4D1A5F-5D47-4666-90B3-FC203DF5316E}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{BE4D1A5F-5D47-4666-90B3-FC203DF5316E}"/>
   </bookViews>
   <sheets>
     <sheet name="Entities" sheetId="1" r:id="rId1"/>

</xml_diff>